<commit_message>
Find the number of rotations
</commit_message>
<xml_diff>
--- a/Data Structures Practice Quizz.xlsx
+++ b/Data Structures Practice Quizz.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://minetgroup-my.sharepoint.com/personal/maureen_chelangat_minet_co_ke/Documents/Desktop/work/dsa-quizzes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="8_{CA6BAA0E-4F43-4947-8FE8-A2A07A3CE697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B969DA91-FB65-4137-8BBC-785AB7EBED71}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{CA6BAA0E-4F43-4947-8FE8-A2A07A3CE697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5CAF0447-953B-4A7B-87C3-D849D4B11DBE}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{5D9121B8-8B25-4864-8004-5AA35198A857}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="14016" windowHeight="13776" xr2:uid="{5D9121B8-8B25-4864-8004-5AA35198A857}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>DATA STRUCTURES</t>
   </si>
@@ -54,21 +54,19 @@
   </si>
   <si>
     <t xml:space="preserve">Given a sorted array of n integers and a target value, determine if the target exists in the array in logarithmic time using the binary search algorithm. If target exists in the array, print the index of it.
-For example, Input: nums[] = [2, 3, 5, 7, 9]target = 7 Output: Element found at index 3  Input: nums[] = [1, 4, 5, 8, 9]target = 2 Output: Element not found. 
+For example, Input: nums[] = [2, 3, 5, 7, 9] target = 7 Output: Element found at index 3  Input: nums[] = [1, 4, 5, 8, 9] target = 2 Output: Element not found. 
 </t>
   </si>
   <si>
-    <t>QUESTION LINK</t>
-  </si>
-  <si>
-    <t>Link</t>
+    <t>Given a circularly sorted integer array, find the total number of times the array is rotated. Assume there are no duplicates in the array, and the rotation is in the anti-clockwise direction.
+For example, Input:  nums = [8, 9, 10, 2, 5, 6] Output: The array is rotated 3 times  Input:  nums = [2, 5, 6, 8, 9, 10] Output: The array is rotated 0 times</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -92,6 +90,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF242323"/>
+      <name val="Nunito"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF242323"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -114,7 +124,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -124,6 +134,15 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -463,16 +482,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E80E17EF-5391-40E8-8DC4-8EA2738A1B29}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="155.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -480,32 +498,38 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="4" t="str">
+      <c r="C2" s="4" t="str">
         <f>HYPERLINK("src/BinarySearch.java", "View Solution")</f>
         <v>View Solution</v>
       </c>
     </row>
+    <row r="3" spans="1:3" ht="45" x14ac:dyDescent="0.3">
+      <c r="A3" s="7"/>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+      <c r="B5" s="5"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B6" s="6"/>
+    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{3A194D1C-404C-4C07-8FDA-DDF5285CEC7D}"/>
-  </hyperlinks>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>